<commit_message>
Fix: MCMA options/correct answers and Kategori statements in questions.json, Quiz_Web_Questions.json, and all Quiz Web files
</commit_message>
<xml_diff>
--- a/Quiz_Web_Bahasa_Indonesia_Paket_1_terbaru.xlsx
+++ b/Quiz_Web_Bahasa_Indonesia_Paket_1_terbaru.xlsx
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan berikut yang TIDAK SESUAI dengan isi teks 'Penyu Sisik: Sang Penjaga Terumbu Karang Nusantara' adalah....</t>
+          <t>Bacalah teks berikut! 'Penyu sisik tergolong hewan reptil yang dilindungi. Cangkangnya bernilai tinggi di pasar hitam, menyebabkan perburuan liar. Tukik (anak penyu) harus dilepas malam hari agar menghindari predator. Konservasi di Derawan dan Sukamade berupaya melindungi populasi ini.' Manakah pernyataan berikut yang merupakan FAKTA? (Pilih lebih dari satu)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -692,22 +692,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Penyu sisik memiliki bentuk paruh runcing menyerupai paruh burung elang.</t>
+          <t>Penyu sisik dilindungi karena populasi menurun akibat perburuan cangkang.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tukik dilepasliarkan pada siang hari terik agar tubuhnya cepat kuat berenang.</t>
+          <t>Tukik dilepas siang hari agar cepat kuat berenang.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Kepulauan Derawan dan Sukamade merupakan contoh lokasi konservasi penyu.</t>
+          <t>Kepulauan Derawan dan Sukamade merupakan lokasi konservasi penyu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Populasi penyu sisik berkurang salah satunya karena perburuan cangkang sisiknya.</t>
+          <t>Cangkang penyu sisik tidak memiliki nilai ekonomis sama sekali.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -722,7 +722,7 @@
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Pada paragraf ketiga dinyatakan: 'Setelah menetas, anak penyu (tukik) dirawat secara intensif selama beberapa hari sebelum akhirnya dilepasliarkan kembali ke laut lepas pada malam atau dini hari guna menghindari serangan burung pemangsa.' Oleh karena itu, pernyataan B (dilepasliarkan pada siang hari terik) tidak sesuai/salah.</t>
+          <t>A: Fakta (teks menyebut perburuan liar karena cangkang bernilai tinggi). B: SALAH, teks menyebut 'malam hari'. C: Fakta (teks menyebut Derawan dan Sukamade). D: SALAH, teks menyebut cangkang 'bernilai tinggi'. Jawaban benar: A, C.</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Latar tempat terjadinya peristiwa penemuan kantong belacu cokelat oleh Arga adalah....</t>
+          <t>Berdasarkan cerita 'Kantong Belacu Cokelat', tentukan kebenaran pernyataan berikut!</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -790,17 +790,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
+          <t>Peristiwa penemuan kantong belacu terjadi di tepi semak rumput gajah dekat jembatan kayu.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
+          <t>Arga menemukan kantong belacu di dalam pasar desa yang ramai.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+          <t>Suasana saat Arga menemukan kantong adalah sunyi dan menegangkan.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -816,7 +816,7 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Pada paragraf pertama tertulis jelas: 'Ketika melewati tikungan jembatan kayu di perbatasan desa, roda depan sepedanya menabrak sesuatu... Di tepi semak-semak rumput gajah, tergeletak sebuah kantong kain belacu berwarna cokelat kusam.' Jadi latar tempatnya adalah B.</t>
+          <t>A: BENAR (teks: 'melewati tikungan jembatan kayu di perbatasan desa... semak rumput gajah'). B: SALAH (bukan di pasar). C: SALAH (suasana tidak sunyi menegangkan, tapi penemuan tak terduga).</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Berdasarkan dialog di atas, keuntungan langsung yang diperoleh siswa ketika menyetorkan sampah anorganik bersih ke Bank Sampah adalah....</t>
+          <t>Berdasarkan dialog Bank Sampah di atas, manakah keuntungan yang diperoleh siswa? (Pilih lebih dari satu)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1021,28 +1021,28 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Mendapatkan nilai rapor tertinggi pada mata pelajaran IPA</t>
+          <t>Mendapatkan saldo tabungan yang bisa ditukar alat tulis atau bibit tanaman.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Memperoleh saldo tabungan yang kelak dapat ditukar dengan alat tulis atau bibit tanaman</t>
+          <t>Belajar menghitung dan mencatat transaksi keuangan sederhana.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Dibebaskan dari tugas piket membersihkan ruang kelas selama satu semester</t>
+          <t>Dibebaskan dari tugas piket membersihkan ruang kelas selamanya.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Diberikan hadiah uang tunai langsung oleh kepala sekolah</t>
+          <t>Mendapatkan hadiah uang tunai langsung dari Kepala Sekolah.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>1, 3</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -1051,7 +1051,7 @@
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Ibu Ratna menjelaskan: 'Pengurus cilik bank sampah akan menimbang... mengonversikannya menjadi saldo tabungan di buku rekening siswa. Saldo tabungan ini pada akhir semester dapat ditukarkan dengan buku tulis, pensil warna, atau bibit tanaman hias.' Pilihan yang tepat adalah B.</t>
+          <t>A: Benar (teks: 'saldo tabungan yang kelak dapat ditukar dengan alat tulis atau bibit tanaman'). B: Benar (implisit dari mengelola tabungan). C: SALAH (tidak disebutkan). D: SALAH (tidak disebutkan). Jawaban benar: A, B.</t>
         </is>
       </c>
     </row>
@@ -1148,15 +1148,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Bacalah petunjuk prosedur berikut untuk menjawab soal nomor 15 dan 16!
-Petunjuk Praktis Menanam Sayuran Hidroponik Sistem Sumbu (Wick System)
-(1) Siapkan botol plastik bekas air mineral ukuran 1,5 liter, lalu potong secara horizontal menjadi dua bagian menggunakan gunting atau *cutter*.
-(2) Buatlah lubang kecil pada tutup botol menggunakan solder atau paku panas, lalu selipkan sehelai kain flanel sepanjang 15 cm sebagai sumbu kapiler.
-(3) Pasang bagian atas botol yang sudah bersumbu ke dalam potongan bagian bawah botol secara terbalik (leher botol menghadap ke dasar).
-(4) [...]
-(5) Masukkan bibit tanaman sawi atau selada yang telah disemai (berdaun 3 sampai 4 helai) dengan hati-hati ke dalam media tanam tersebut.
-(6) Tuangkan larutan nutrisi hidroponik (larutan AB Mix) ke dalam wadah bagian bawah hingga menyentuh separuh sumbu flanel, lalu letakkan di area yang terkena sinar matahari cukup.
-Kalimat yang paling tepat dan runtut untuk melengkapi langkah nomor (4) pada petunjuk hidroponik tersebut adalah....</t>
+          <t>Berdasarkan prosedur menanam sawi hidroponik, tentukan kebenaran!</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1166,17 +1158,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
+          <t>Botol plastik bagian bawah digunakan sebagai wadah nutrisi.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
+          <t>Biji benih sawi direndam air hangat selama 2 hari sebelum ditanam.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+          <t>Media tanam yang digunakan adalah arang sekam atau rockwool.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1192,7 +1184,7 @@
       <c r="J16" s="3" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Setelah memasang bagian botol secara terbalik dengan sumbu (langkah 3) dan sebelum menempatkan bibit bertunas (langkah 5), wadah harus diisi media tanam (seperti arang sekam, cocopeat, atau rockwool). Kalimat B adalah langkah yang logis dan tepat.</t>
+          <t>A: BENAR (botol bawah jadi wadah nutrisi). B: SALAH (benih direndam air biasa, bukan hangat 2 hari). C: BENAR (teks: 'arang sekam atau rockwool').</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1286,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Perhatikan kalimat-kalimat petunjuk pembuatan puding berikut!
-(1) Setelah uap panasnya berkurang, masukkan puding ke dalam lemari es hingga mengeras.
-(2) Campurkan bubuk agar-agar, gula pasir, dan air kelapa muda ke dalam panci secara merata.
-(3) Rebus adonan di atas api sedang sambil terus diaduk perlahan hingga mendidih sempurna.
-(4) Tuangkan cairan puding yang telah mendidih ke dalam cetakan yang telah disiapkan.
-Urutan petunjuk yang tepat dan logis agar menjadi teks prosedur yang padu adalah....</t>
+          <t>Perhatikan kalimat acak berikut! (1) Tuang adonan ke cetakan. (2) Campur tepung, gula, telur, dan santan. (3) Kukus selama 20 menit. (4) Aduk hingga rata. Urutan yang tepat adalah.... (Pilih lebih dari satu yang benar)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1309,28 +1296,28 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>(2) - (3) - (4) - (1)</t>
+          <t>Urutan logis dimulai dari mencampur bahan (2).</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>(2) - (4) - (3) - (1)</t>
+          <t>Pengadukan (4) dilakukan setelah mencampur (2).</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>(3) - (2) - (4) - (1)</t>
+          <t>Mengukus (3) dilakukan sebelum menuang ke cetakan (1).</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>(3) - (4) - (2) - (1)</t>
+          <t>Urutan lengkapnya adalah (2) - (4) - (1) - (3).</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>1, 3</t>
+          <t>1, 2, 4</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
@@ -1339,12 +1326,7 @@
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Urutan memasak puding yang logis:
-- (2) Campurkan bahan ke panci.
-- (3) Rebus di atas api sambil diaduk hingga mendidih.
-- (4) Tuangkan ke cetakan.
-- (1) Masukkan ke lemari es hingga mengeras.
-Urutan yang tepat adalah (2) - (3) - (4) - (1) (Pilihan A).</t>
+          <t>Urutan: (2) Campur -&gt; (4) Aduk -&gt; (1) Tuang cetakan -&gt; (3) Kukus. A: Benar. B: Benar. C: SALAH (mengukus SETELAH tuang cetakan). D: Benar (urutan lengkap benar). Jawaban benar: A, B, D.</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1383,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Penulisan kalimat langsung berikut yang menggunakan tanda baca dan huruf kapital secara tepat adalah....</t>
+          <t>Perhatikan kalimat langsung berikut! Tentukan kebenaran penulisan tanda baca &amp; huruf kapital.</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1411,17 +1393,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
+          <t>Kalimat: Ibu berpesan, "Tolong rapikan buku pelajaran di mejamu, Farhan!" → Penulisan BENAR.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
+          <t>Kalimat: Ibu berpesan: "tolong rapikan buku pelajaran di mejamu, Farhan!" → Penulisan BENAR.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+          <t>Kalimat: Ibu berpesan, "Tolong rapikan buku pelajaran di mejamu Farhan"! → Penulisan BENAR.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1437,11 +1419,7 @@
       <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Aturan penulisan kalimat langsung:
-1. Pengiring diikuti tanda koma (,).
-2. Kalimat petikan diawali huruf kapital di dalam tanda petik (").
-3. Tanda seru (!) atau tanda titik diletakkan SEBELUM tanda petik penutup (").
-Jadi penulisan yang benar adalah: Ibu berpesan, "Tolong rapikan buku pelajaran di mejamu, Farhan!" (Pilihan A).</t>
+          <t>A: BENAR (komi pengiring, kapital awal petik, tanda baca di dalam petik). B: SALAH (huruf 't' dalam petik harus kapital). C: SALAH (tanda seru harus di dalam petik, 'Farhan' kurang koma).</t>
         </is>
       </c>
     </row>

</xml_diff>